<commit_message>
updated files after test run on 0.3k
test run on 0.3k and made some changes . also updated other files to be in sync with general folder
</commit_message>
<xml_diff>
--- a/Metadata/Helium Refill.xlsx
+++ b/Metadata/Helium Refill.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="107">
   <si>
     <t>Date</t>
   </si>
@@ -351,6 +351,12 @@
   </si>
   <si>
     <t>15/5/2024</t>
+  </si>
+  <si>
+    <t>150 the system dewar</t>
+  </si>
+  <si>
+    <t>21/1/2025</t>
   </si>
 </sst>
 </file>
@@ -7524,7 +7530,7 @@
     </row>
     <row r="150" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="2">
-        <v>45296</v>
+        <v>45413</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>44</v>
@@ -7627,14 +7633,22 @@
       <c r="AC151" s="1"/>
     </row>
     <row r="152" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="1"/>
-      <c r="B152" s="1"/>
+      <c r="A152" s="2">
+        <v>45636</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="C152" s="1"/>
       <c r="D152" s="1"/>
-      <c r="E152" s="1"/>
+      <c r="E152" s="1" t="s">
+        <v>105</v>
+      </c>
       <c r="F152" s="1"/>
       <c r="G152" s="1"/>
-      <c r="H152" s="1"/>
+      <c r="H152" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I152" s="1"/>
       <c r="J152" s="1"/>
       <c r="K152" s="1"/>
@@ -7658,16 +7672,37 @@
       <c r="AC152" s="1"/>
     </row>
     <row r="153" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="1"/>
-      <c r="B153" s="1"/>
-      <c r="C153" s="1"/>
-      <c r="D153" s="1"/>
-      <c r="E153" s="1"/>
-      <c r="F153" s="1"/>
-      <c r="G153" s="1"/>
-      <c r="H153" s="1"/>
-      <c r="I153" s="1"/>
-      <c r="J153" s="1"/>
+      <c r="A153" s="2">
+        <v>45652</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C153" s="1">
+        <v>22.2</v>
+      </c>
+      <c r="D153" s="1">
+        <v>149.34</v>
+      </c>
+      <c r="E153" s="1">
+        <v>140</v>
+      </c>
+      <c r="F153" s="1">
+        <v>4861.4030000000002</v>
+      </c>
+      <c r="G153" s="1">
+        <v>4872.74</v>
+      </c>
+      <c r="H153" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I153" s="1">
+        <v>15.1122</v>
+      </c>
+      <c r="J153" s="1">
+        <f xml:space="preserve"> D153+I153-C153</f>
+        <v>142.25220000000002</v>
+      </c>
       <c r="K153" s="1"/>
       <c r="L153" s="1"/>
       <c r="M153" s="1"/>
@@ -7689,16 +7724,37 @@
       <c r="AC153" s="1"/>
     </row>
     <row r="154" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="1"/>
-      <c r="B154" s="1"/>
-      <c r="C154" s="1"/>
-      <c r="D154" s="1"/>
-      <c r="E154" s="1"/>
-      <c r="F154" s="1"/>
-      <c r="G154" s="1"/>
-      <c r="H154" s="1"/>
-      <c r="I154" s="1"/>
-      <c r="J154" s="1"/>
+      <c r="A154" s="2">
+        <v>45665</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C154" s="1">
+        <v>42</v>
+      </c>
+      <c r="D154" s="1">
+        <v>150.5</v>
+      </c>
+      <c r="E154" s="1">
+        <v>120</v>
+      </c>
+      <c r="F154" s="1">
+        <v>4954.8710000000001</v>
+      </c>
+      <c r="G154" s="1">
+        <v>4964.42</v>
+      </c>
+      <c r="H154" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I154" s="1">
+        <v>12.7288</v>
+      </c>
+      <c r="J154" s="1">
+        <f xml:space="preserve"> D154+I154-C154</f>
+        <v>121.22880000000001</v>
+      </c>
       <c r="K154" s="1"/>
       <c r="L154" s="1"/>
       <c r="M154" s="1"/>
@@ -7720,16 +7776,37 @@
       <c r="AC154" s="1"/>
     </row>
     <row r="155" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="1"/>
-      <c r="B155" s="1"/>
-      <c r="C155" s="1"/>
-      <c r="D155" s="1"/>
-      <c r="E155" s="1"/>
-      <c r="F155" s="1"/>
-      <c r="G155" s="1"/>
-      <c r="H155" s="1"/>
-      <c r="I155" s="1"/>
-      <c r="J155" s="1"/>
+      <c r="A155" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C155" s="1">
+        <v>43.4</v>
+      </c>
+      <c r="D155" s="1">
+        <v>139.77000000000001</v>
+      </c>
+      <c r="E155" s="1">
+        <v>110</v>
+      </c>
+      <c r="F155" s="1">
+        <v>5049.0389999999998</v>
+      </c>
+      <c r="G155" s="1">
+        <v>5060.8</v>
+      </c>
+      <c r="H155" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I155" s="1">
+        <v>15.6774</v>
+      </c>
+      <c r="J155" s="1">
+        <f xml:space="preserve"> D155+I155-C155</f>
+        <v>112.04740000000001</v>
+      </c>
       <c r="K155" s="1"/>
       <c r="L155" s="1"/>
       <c r="M155" s="1"/>

</xml_diff>